<commit_message>
Actualización de proveedores mayo 2026
</commit_message>
<xml_diff>
--- a/backend/rutas_manuales.xlsx
+++ b/backend/rutas_manuales.xlsx
@@ -409,10 +409,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aduana San Bartolo, Ilopango Soyapango</v>
+        <v>Aduana San Bartolo, Ilopango, Soyapango</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-06T16:57:03.652Z</v>
+        <v>2026-05-12T19:42:22.061Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>